<commit_message>
chore: run build script for masp profile
</commit_message>
<xml_diff>
--- a/profiles/ro-crate-masp/profile-crate/ro-crate-metadata.xlsx
+++ b/profiles/ro-crate-masp/profile-crate/ro-crate-metadata.xlsx
@@ -146,7 +146,7 @@
     <t>"https://language-research-technology.github.io/ro-crate-masp/profiles/ro-crate-masp/profile-crate/"</t>
   </si>
   <si>
-    <t>2026-07-22T15:37:00+10:00</t>
+    <t>2026-08-13T17:08:55+02:00</t>
   </si>
   <si>
     <t>profile-documentation.md</t>
@@ -164,7 +164,7 @@
     <t>["https://www.nationalarchives.gov.uk/PRONOM/fmt/817", application/json]</t>
   </si>
   <si>
-    <t>2026-05-22T08:29:17+10:00</t>
+    <t>2026-08-13T15:49:27+02:00</t>
   </si>
   <si>
     <t>Mini Crate-O mode file for this profile (metadata, input groups, lookup and enabled classes — the schema/grammar is provided by the MASP profile crate itself).</t>
@@ -443,7 +443,7 @@
     <t>"#class_MetadataDescriptor"</t>
   </si>
   <si>
-    <t>["Text", "#propertyValue_prop_id_MetadataDescriptor"]</t>
+    <t>"#propertyValue_prop_id_MetadataDescriptor"</t>
   </si>
   <si>
     <t>#prop_conformsTo_MetadataDescriptor</t>
@@ -779,12 +779,18 @@
     <t>Canonical identifiers that indicate conformance to this profile.</t>
   </si>
   <si>
+    <t>https://www.nationalarchives.gov.uk/PRONOM/fmt/471</t>
+  </si>
+  <si>
+    <t>DigitalFormat</t>
+  </si>
+  <si>
+    <t>Hypertext Markup Language</t>
+  </si>
+  <si>
     <t>https://www.nationalarchives.gov.uk/PRONOM/fmt/1149</t>
   </si>
   <si>
-    <t>DigitalFormat</t>
-  </si>
-  <si>
     <t>Markdown</t>
   </si>
   <si>
@@ -792,12 +798,6 @@
   </si>
   <si>
     <t>JSON Data Interchange Format</t>
-  </si>
-  <si>
-    <t>https://www.nationalarchives.gov.uk/PRONOM/fmt/471</t>
-  </si>
-  <si>
-    <t>Hypertext Markup Language</t>
   </si>
 </sst>
 </file>
@@ -2865,6 +2865,9 @@
       <c r="E23" t="s">
         <v>200</v>
       </c>
+      <c r="H23">
+        <v>1</v>
+      </c>
       <c r="I23" t="s">
         <v>209</v>
       </c>

</xml_diff>

<commit_message>
fix: add maxCounts as per #23
</commit_message>
<xml_diff>
--- a/profiles/ro-crate-masp/profile-crate/ro-crate-metadata.xlsx
+++ b/profiles/ro-crate-masp/profile-crate/ro-crate-metadata.xlsx
@@ -146,7 +146,7 @@
     <t>"https://language-research-technology.github.io/ro-crate-masp/profiles/ro-crate-masp/profile-crate/"</t>
   </si>
   <si>
-    <t>2026-08-13T17:18:39+02:00</t>
+    <t>2026-08-13T17:26:40+02:00</t>
   </si>
   <si>
     <t>profile-documentation.md</t>
@@ -2683,6 +2683,9 @@
       <c r="F16" t="s">
         <v>149</v>
       </c>
+      <c r="H16">
+        <v>1</v>
+      </c>
       <c r="I16" t="s">
         <v>187</v>
       </c>
@@ -2732,6 +2735,9 @@
       <c r="F18" t="s">
         <v>193</v>
       </c>
+      <c r="H18">
+        <v>1</v>
+      </c>
       <c r="I18" t="s">
         <v>194</v>
       </c>
@@ -2758,6 +2764,9 @@
       <c r="F19" t="s">
         <v>193</v>
       </c>
+      <c r="H19">
+        <v>1</v>
+      </c>
       <c r="I19" t="s">
         <v>197</v>
       </c>
@@ -2894,6 +2903,9 @@
       <c r="F24" t="s">
         <v>193</v>
       </c>
+      <c r="H24">
+        <v>1</v>
+      </c>
       <c r="I24" t="s">
         <v>211</v>
       </c>
@@ -2919,6 +2931,9 @@
       </c>
       <c r="F25" t="s">
         <v>193</v>
+      </c>
+      <c r="H25">
+        <v>1</v>
       </c>
       <c r="I25" t="s">
         <v>213</v>

</xml_diff>